<commit_message>
Forjar: ajustes de contenido del cliente y diagrama de equipo desde Excel
</commit_message>
<xml_diff>
--- a/datos/directorio_forjar.xlsx
+++ b/datos/directorio_forjar.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carol\CH_projects\SDIS\Gestion de conocimiento\gestor-conocimiento-2025\datos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mi unidad\CH_projects\SDIS\Gestion de conocimiento\gestor-conocimiento-2025\datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C37A85F-FE3A-4898-A8ED-0BAEF679935F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CC30506-4E51-414A-81B8-742C03E184F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -67,13 +67,13 @@
     <t>https://maps.app.goo.gl/W7w7Ck5WoxRwzpYx8</t>
   </si>
   <si>
-    <t>https://maps.app.goo.gl/oAztqaBt9KPS97cn9</t>
-  </si>
-  <si>
     <t>Carrera 44 # 58 C - 90 Sur</t>
   </si>
   <si>
-    <t>Carrera 12G # 22B-29 Sur</t>
+    <t>Carrera 12G # 22B - 61 Sur</t>
+  </si>
+  <si>
+    <t>https://maps.app.goo.gl/Woccs9GMfvdKQrDs7</t>
   </si>
 </sst>
 </file>
@@ -516,7 +516,7 @@
         <v>9</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D3" s="3">
         <v>4.5752065189313402</v>
@@ -536,22 +536,21 @@
         <v>10</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="3">
+        <v>4.5789965257665903</v>
+      </c>
+      <c r="E4" s="3">
+        <v>-74.1019230983417</v>
+      </c>
+      <c r="F4" s="5" t="s">
         <v>17</v>
-      </c>
-      <c r="D4" s="3">
-        <v>4.57935554987393</v>
-      </c>
-      <c r="E4" s="3">
-        <v>-74.101570213492707</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>15</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="F3" r:id="rId1" xr:uid="{69B84CFC-6E9A-4755-8326-97A389574060}"/>
-    <hyperlink ref="F4" r:id="rId2" xr:uid="{87D5CA30-10A3-4A9F-87C4-D55E5AB722C1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>